<commit_message>
docs: pin test baseline and start profile reviews
</commit_message>
<xml_diff>
--- a/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
+++ b/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb14d52f710be419b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="R82076cf7eab245a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R57c7d5f6c12c45c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="R325a6d1b41b247f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -478,7 +478,7 @@
         <x:v>Register evidence level</x:v>
       </x:c>
       <x:c r="B14" s="15" t="str">
-        <x:v>Six per-row evidence/decision fields have been added to the register. Row-level reviews, feature assignments, and final dispositions remain pending.</x:v>
+        <x:v>The first six framework entries have source/metadata notes and provisional use boundaries; deeper API/runtime checks remain open, and the other 288 entries still need source review.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -502,7 +502,7 @@
         <x:v>Current RWT boundary</x:v>
       </x:c>
       <x:c r="B17" s="15" t="str">
-        <x:v>The local client/server package IDs and order match in this snapshot, but server enforcement is disabled and its build hash is unresolved. Official release notes are not proof that this local server runs that release. Custom transfers and scenario joining remain untested.</x:v>
+        <x:v>The 294 local client/server IDs and order match, but the server does not enforce them. The Windows server archive matches the published RWT 26.8.31.1 asset; the client DLL is pinned separately. Custom transfers, visits, and scenario joining remain untested.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1090,37 +1090,37 @@
         <x:v>Mod framework</x:v>
       </x:c>
       <x:c r="G2" s="24" t="str">
-        <x:v>Required by RimWorld Together and Vanilla Expanded Framework in their published listings.</x:v>
+        <x:v>Listed as a dependency by RWT and several selected frameworks. Rimrooms requires it only for the selected co-op path, not solo Core play.</x:v>
       </x:c>
       <x:c r="H2" s="24" t="str">
-        <x:v>Keep the framework available for the profile's dependent mods. Reuse public APIs only when a specific Backrooms integration needs them; the company mod must not duplicate framework services.</x:v>
+        <x:v>Keep the shared library available for dependent co-op/profile mods. Add a Rimrooms patch only if a specific feature needs one.</x:v>
       </x:c>
       <x:c r="I2" s="24" t="str">
-        <x:v>Load before consuming mods. Verify the exact 1.6 package version and transitive dependencies; avoid making a framework a Backrooms core requirement without a concrete integration.</x:v>
+        <x:v>Preserve the required load-before-Core order; record both local metadata and active assembly identities because their version strings differ.</x:v>
       </x:c>
       <x:c r="J2" s="24" t="str">
-        <x:v>Low to medium: pin the exact 1.6 build and dependency order; consume public APIs only when an integration needs them.</x:v>
+        <x:v>Retest the dependency order if Harmony or a dependent RWT build changes.</x:v>
       </x:c>
       <x:c r="K2" s="24" t="str">
-        <x:v>Required by the official RWT and VEF listings; exact local build still needs pinning.</x:v>
+        <x:v>Workshop description and installed metadata reviewed; source/API and runtime checks pending.</x:v>
       </x:c>
       <x:c r="L2" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-MP;RR-COMPAT</x:v>
       </x:c>
       <x:c r="M2" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/2009463077-brrainz.harmony.md</x:v>
       </x:c>
       <x:c r="N2" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Workshop and installed metadata reviewed; Rimrooms compatibility pending</x:v>
       </x:c>
       <x:c r="O2" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: required only for the selected RWT co-op path; optional for solo Core play.</x:v>
       </x:c>
       <x:c r="P2" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; metadata 2.4.2.0; active DLL 2.4.1.0+789df191bbaf6610232d50e7ef7dddc0d2812549</x:v>
       </x:c>
       <x:c r="Q2" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; pinned co-op profile check pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="45" customHeight="1">
@@ -1555,37 +1555,37 @@
         <x:v>Mod framework</x:v>
       </x:c>
       <x:c r="G11" s="24" t="str">
-        <x:v>Selected profile framework; not a Backrooms core dependency.</x:v>
+        <x:v>Harmony required; optional storage framework in this profile, not a Rimrooms core dependency.</x:v>
       </x:c>
       <x:c r="H11" s="24" t="str">
-        <x:v>Keep the framework available for the profile's dependent mods. Reuse public APIs only when a specific Backrooms integration needs them; the company mod must not duplicate framework services.</x:v>
+        <x:v>Consider standard interoperability for facility stock and recovered evidence only if it improves the player's existing storage workflow.</x:v>
       </x:c>
       <x:c r="I11" s="24" t="str">
-        <x:v>Load before consuming mods. Verify the exact 1.6 package version and transitive dependencies; avoid making a framework a Backrooms core requirement without a concrete integration.</x:v>
+        <x:v>Use a narrow bridge only for a reproduced storage need; keep vanilla stockpiles useful when ASF is absent.</x:v>
       </x:c>
       <x:c r="J11" s="24" t="str">
-        <x:v>Low to medium: pin the exact 1.6 build and dependency order; consume public APIs only when an integration needs them.</x:v>
+        <x:v>Test item filters, display, and temperature only if an integration is selected.</x:v>
       </x:c>
       <x:c r="K11" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
+        <x:v>Workshop description/change notes and local About.xml reviewed; exact API and runtime interactions pending.</x:v>
       </x:c>
       <x:c r="L11" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-FAC;RR-EVD;RR-COMPAT</x:v>
       </x:c>
       <x:c r="M11" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/3033901359-adaptive.storage.framework.md</x:v>
       </x:c>
       <x:c r="N11" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Workshop, change notes, and installed metadata reviewed; compatibility pending</x:v>
       </x:c>
       <x:c r="O11" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: optional storage interoperability; no Rimrooms core dependency planned.</x:v>
       </x:c>
       <x:c r="P11" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; local About.xml lists 1.6 support; no modVersion stated</x:v>
       </x:c>
       <x:c r="Q11" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; custom storage/evidence behavior pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="45" customHeight="1">
@@ -1608,37 +1608,37 @@
         <x:v>Mod framework</x:v>
       </x:c>
       <x:c r="G12" s="24" t="str">
-        <x:v>Selected profile framework; not a Backrooms core dependency.</x:v>
+        <x:v>Harmony required; the framework adds no vehicles by itself and is not a Rimrooms core dependency.</x:v>
       </x:c>
       <x:c r="H12" s="24" t="str">
-        <x:v>Keep the framework available for the profile's dependent mods. Reuse public APIs only when a specific Backrooms integration needs them; the company mod must not duplicate framework services.</x:v>
+        <x:v>Consider future vehicle-based expedition or outpost support only if it fits Odyssey/Gravship Expanded and verified RWT travel.</x:v>
       </x:c>
       <x:c r="I12" s="24" t="str">
-        <x:v>Load before consuming mods. Verify the exact 1.6 package version and transitive dependencies; avoid making a framework a Backrooms core requirement without a concrete integration.</x:v>
+        <x:v>Keep the machine gate as the Backrooms entry point and preserve native gravship behavior; do not add vehicles solely because the framework is installed.</x:v>
       </x:c>
       <x:c r="J12" s="24" t="str">
-        <x:v>Low to medium: pin the exact 1.6 build and dependency order; consume public APIs only when an integration needs them.</x:v>
+        <x:v>Local metadata lists RimThreaded as incompatible; vehicle, save, and multiplayer interactions are untested.</x:v>
       </x:c>
       <x:c r="K12" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
+        <x:v>Workshop description and local About.xml reviewed; vehicle, save, and multiplayer interactions pending.</x:v>
       </x:c>
       <x:c r="L12" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-OUT;RR-SPACEFLIGHT;RR-COMPAT</x:v>
       </x:c>
       <x:c r="M12" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/3014915404-SmashPhil.VehicleFramework.md</x:v>
       </x:c>
       <x:c r="N12" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Workshop and installed metadata reviewed; compatibility pending</x:v>
       </x:c>
       <x:c r="O12" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: optional vehicle interoperability only if it fits expeditions/outposts and the gravship plan.</x:v>
       </x:c>
       <x:c r="P12" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; Vehicle Framework 1.6.2144</x:v>
       </x:c>
       <x:c r="Q12" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; vehicle/RWT travel behavior pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="45" customHeight="1">
@@ -1661,37 +1661,37 @@
         <x:v>Mod framework</x:v>
       </x:c>
       <x:c r="G13" s="24" t="str">
-        <x:v>Selected profile framework; not a Backrooms core dependency.</x:v>
+        <x:v>Harmony required; optional profile XML tool and not a Rimrooms core dependency.</x:v>
       </x:c>
       <x:c r="H13" s="24" t="str">
-        <x:v>Keep the framework available for the profile's dependent mods. Reuse public APIs only when a specific Backrooms integration needs them; the company mod must not duplicate framework services.</x:v>
+        <x:v>Revisit only if a real feature needs a documented XML patch or settings operation.</x:v>
       </x:c>
       <x:c r="I13" s="24" t="str">
-        <x:v>Load before consuming mods. Verify the exact 1.6 package version and transitive dependencies; avoid making a framework a Backrooms core requirement without a concrete integration.</x:v>
+        <x:v>Keep core definitions and settings independent; no custom XML Extensions operation selected.</x:v>
       </x:c>
       <x:c r="J13" s="24" t="str">
-        <x:v>Low to medium: pin the exact 1.6 build and dependency order; consume public APIs only when an integration needs them.</x:v>
+        <x:v>Check load order and patches only if Rimrooms adopts a documented operation.</x:v>
       </x:c>
       <x:c r="K13" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
+        <x:v>Workshop description and local About.xml reviewed; operation/API and runtime checks pending.</x:v>
       </x:c>
       <x:c r="L13" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-COMPAT</x:v>
       </x:c>
       <x:c r="M13" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/2574315206-imranfish.xmlextensions.md</x:v>
       </x:c>
       <x:c r="N13" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Workshop and installed metadata reviewed; specific API use pending</x:v>
       </x:c>
       <x:c r="O13" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: optional profile tool; no Rimrooms dependency planned.</x:v>
       </x:c>
       <x:c r="P13" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; local About.xml lists 1.6 support; no modVersion stated</x:v>
       </x:c>
       <x:c r="Q13" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; no custom XML Extensions use selected.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="45" customHeight="1">
@@ -1714,37 +1714,37 @@
         <x:v>Mod framework</x:v>
       </x:c>
       <x:c r="G14" s="24" t="str">
-        <x:v>Selected profile framework; not a Backrooms core dependency.</x:v>
+        <x:v>Harmony required; optional shared library used by profile mods, not a Rimrooms core dependency.</x:v>
       </x:c>
       <x:c r="H14" s="24" t="str">
-        <x:v>Keep the framework available for the profile's dependent mods. Reuse public APIs only when a specific Backrooms integration needs them; the company mod must not duplicate framework services.</x:v>
+        <x:v>Leave existing HugsLib-dependent mods usable; treat shared logs as support evidence when supplied by a player.</x:v>
       </x:c>
       <x:c r="I14" s="24" t="str">
-        <x:v>Load before consuming mods. Verify the exact 1.6 package version and transitive dependencies; avoid making a framework a Backrooms core requirement without a concrete integration.</x:v>
+        <x:v>Do not require HugsLib services or log upload for campaign play; preserve the local after-Core load order.</x:v>
       </x:c>
       <x:c r="J14" s="24" t="str">
-        <x:v>Low to medium: pin the exact 1.6 build and dependency order; consume public APIs only when an integration needs them.</x:v>
+        <x:v>Confirm startup and support-log flow on the eventual clean and selected mod profiles.</x:v>
       </x:c>
       <x:c r="K14" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
+        <x:v>Workshop description and local About.xml reviewed; Rimrooms service and runtime interactions pending.</x:v>
       </x:c>
       <x:c r="L14" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-COMPAT</x:v>
       </x:c>
       <x:c r="M14" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/818773962-UnlimitedHugs.HugsLib.md</x:v>
       </x:c>
       <x:c r="N14" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Workshop and installed metadata reviewed; compatibility pending</x:v>
       </x:c>
       <x:c r="O14" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: optional profile library; no direct Rimrooms dependency planned.</x:v>
       </x:c>
       <x:c r="P14" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; local description version 12.0.0</x:v>
       </x:c>
       <x:c r="Q14" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; no direct Rimrooms service use selected.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="45" customHeight="1">
@@ -1767,37 +1767,37 @@
         <x:v>Mod framework</x:v>
       </x:c>
       <x:c r="G15" s="24" t="str">
-        <x:v>Required when either selected Vanilla Gravship Expanded chapter is enabled.</x:v>
+        <x:v>Harmony required; dependency of the selected Gravship Expanded chapters and optional to the Core-only campaign.</x:v>
       </x:c>
       <x:c r="H15" s="24" t="str">
-        <x:v>Keep the framework available for the profile's dependent mods. Reuse public APIs only when a specific Backrooms integration needs them; the company mod must not duplicate framework services.</x:v>
+        <x:v>Retain it for the chosen late-game gravship chain; use its services only through a selected, documented dependency.</x:v>
       </x:c>
       <x:c r="I15" s="24" t="str">
-        <x:v>Load before consuming mods. Verify the exact 1.6 package version and transitive dependencies; avoid making a framework a Backrooms core requirement without a concrete integration.</x:v>
+        <x:v>Keep gravship content behind the DLC/mod boundary; preserve a complete gate campaign without VEF or Odyssey.</x:v>
       </x:c>
       <x:c r="J15" s="24" t="str">
-        <x:v>Low to medium: pin the exact 1.6 build and dependency order; consume public APIs only when an integration needs them.</x:v>
+        <x:v>Local metadata lists RangeAnimalFramework as incompatible; check it against the final 294 profile and VGE warnings.</x:v>
       </x:c>
       <x:c r="K15" s="24" t="str">
-        <x:v>Official Workshop description and dependency listing reviewed.</x:v>
+        <x:v>Workshop description and local About.xml reviewed; specific API, gravship conflicts, and combined-profile behavior pending.</x:v>
       </x:c>
       <x:c r="L15" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-SPACEFLIGHT;RR-COMPAT</x:v>
       </x:c>
       <x:c r="M15" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/2023507013-OskarPotocki.VanillaFactionsExpanded.Core.md</x:v>
       </x:c>
       <x:c r="N15" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Workshop and installed metadata reviewed; VGE runtime checks pending</x:v>
       </x:c>
       <x:c r="O15" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: required by the selected Gravship Expanded chain; optional to the Core-only Rimrooms campaign.</x:v>
       </x:c>
       <x:c r="P15" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; local About.xml lists 1.6 support; no modVersion stated</x:v>
       </x:c>
       <x:c r="Q15" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; clean VGE and combined-profile checks pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="45" customHeight="1">
@@ -16643,7 +16643,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02fc116f69be48fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b108bc1453f48af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: sync mod reviews and source handoff paths
</commit_message>
<xml_diff>
--- a/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
+++ b/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R57c7d5f6c12c45c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="R325a6d1b41b247f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R33055fb13a884bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="R15bfcc9aaae54e2b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -478,7 +478,7 @@
         <x:v>Register evidence level</x:v>
       </x:c>
       <x:c r="B14" s="15" t="str">
-        <x:v>The first six framework entries have source/metadata notes and provisional use boundaries; deeper API/runtime checks remain open, and the other 288 entries still need source review.</x:v>
+        <x:v>Twelve profile rows have source/metadata notes and provisional use boundaries; API/runtime checks remain open, and the other 282 entries need their first source review.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -690,7 +690,7 @@
         <x:v>Materials, cargo, and recovered resources</x:v>
       </x:c>
       <x:c r="B41" s="17" t="n">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -834,7 +834,7 @@
         <x:v>Staff work-flow quality of life</x:v>
       </x:c>
       <x:c r="B59" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -1111,13 +1111,13 @@
         <x:v>docs/research/reviews/mods/2009463077-brrainz.harmony.md</x:v>
       </x:c>
       <x:c r="N2" s="27" t="str">
-        <x:v>Workshop and installed metadata reviewed; Rimrooms compatibility pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O2" s="27" t="str">
         <x:v>Provisional: required only for the selected RWT co-op path; optional for solo Core play.</x:v>
       </x:c>
       <x:c r="P2" s="27" t="str">
-        <x:v>RimWorld 1.6.4871 rev590; metadata 2.4.2.0; active DLL 2.4.1.0+789df191bbaf6610232d50e7ef7dddc0d2812549</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; Harmony About.xml 2.4.2.0; active DLL product 2.4.1.0+789df191bbaf6610232d50e7ef7dddc0d2812549</x:v>
       </x:c>
       <x:c r="Q2" s="27" t="str">
         <x:v>Not runtime tested; pinned co-op profile check pending.</x:v>
@@ -1143,37 +1143,37 @@
         <x:v>Staff psychology, relationships, and faction standing</x:v>
       </x:c>
       <x:c r="G3" s="24" t="str">
-        <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
+        <x:v>Selected profile entry; changes pawn mood/opinion rules but is not a Rimrooms dependency.</x:v>
       </x:c>
       <x:c r="H3" s="24" t="str">
-        <x:v>Use the active trait, memory, social-fight, relationship, conversion, and faction-reaction rules when generating applicants, workplace incidents, and crew histories. Keep the company's evaluation based on actual pawn traits, skills, and relationships.</x:v>
+        <x:v>Let staff keep the profile's own reactions. Avoid making Rimrooms progression depend on its specific mood balance.</x:v>
       </x:c>
       <x:c r="I3" s="24" t="str">
-        <x:v>Medium: these mods change the staff and visitor experience. Avoid replacing their thought, relation, or faction logic; check how hostility and guest incidents affect company reputation.</x:v>
+        <x:v>Keep any future company thoughts isolated and additive; do not overwrite its thought definitions.</x:v>
       </x:c>
       <x:c r="J3" s="24" t="str">
-        <x:v>Low to medium: preserve native jobs, needs, guest/faction ownership, and social behavior; test custom role suggestions around them.</x:v>
+        <x:v>Local and Workshop metadata stop at RimWorld 1.4; its page warns about ThoughtDef overrides and load order.</x:v>
       </x:c>
       <x:c r="K3" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
+        <x:v>Workshop page and installed metadata reviewed; declared support stops at 1.4; 1.6 compatibility pending.</x:v>
       </x:c>
       <x:c r="L3" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-STA;RR-COMPAT</x:v>
       </x:c>
       <x:c r="M3" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/1543063349-SF.Grim.Reality.md</x:v>
       </x:c>
       <x:c r="N3" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O3" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: retain as a selected-profile compatibility case; do not depend on its thought balance until 1.6 support is demonstrated.</x:v>
       </x:c>
       <x:c r="P3" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; local metadata lists RimWorld 1.0-1.4</x:v>
       </x:c>
       <x:c r="Q3" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; mood/thought and social behavior with five DLC and profile mods pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="45" customHeight="1">
@@ -1196,37 +1196,37 @@
         <x:v>Interface, scenario setup, and quality of life</x:v>
       </x:c>
       <x:c r="G4" s="24" t="str">
-        <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
+        <x:v>Harmony required; optional startup/support utility and not a Rimrooms gameplay dependency.</x:v>
       </x:c>
       <x:c r="H4" s="24" t="str">
-        <x:v>Preserve the mod's interface or scenario convenience. The Backrooms Operations board should add a focused company view and link to existing vanilla/mod tabs instead of replacing unrelated menus.</x:v>
+        <x:v>Preserve its existing progress display for startup, map generation, and save loading.</x:v>
       </x:c>
       <x:c r="I4" s="24" t="str">
-        <x:v>Low: avoid patching visual-only or convenience features. Scenario editors may be useful for development but must not become a runtime dependency or a campaign progression requirement.</x:v>
+        <x:v>No Rimrooms screen or startup patch planned.</x:v>
       </x:c>
       <x:c r="J4" s="24" t="str">
-        <x:v>Low: avoid overriding hotkeys, scenario controls, or unrelated vanilla tabs.</x:v>
+        <x:v>Harmony/load order; page lists conflicts with RimThemes and Startup Impact Continued. Neither appears in current inventory names/IDs.</x:v>
       </x:c>
       <x:c r="K4" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
+        <x:v>Official Workshop page and installed metadata reviewed; startup compatibility pending.</x:v>
       </x:c>
       <x:c r="L4" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-COMPAT</x:v>
       </x:c>
       <x:c r="M4" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/3535481557-ilyvion.LoadingProgress.md</x:v>
       </x:c>
       <x:c r="N4" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O4" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: optional support utility; no Rimrooms runtime dependency.</x:v>
       </x:c>
       <x:c r="P4" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; Loading Progress 0.16.0</x:v>
       </x:c>
       <x:c r="Q4" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; exact profile startup and named conflicts pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="45" customHeight="1">
@@ -1576,13 +1576,13 @@
         <x:v>docs/research/reviews/mods/3033901359-adaptive.storage.framework.md</x:v>
       </x:c>
       <x:c r="N11" s="27" t="str">
-        <x:v>Workshop, change notes, and installed metadata reviewed; compatibility pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O11" s="27" t="str">
         <x:v>Provisional: optional storage interoperability; no Rimrooms core dependency planned.</x:v>
       </x:c>
       <x:c r="P11" s="27" t="str">
-        <x:v>RimWorld 1.6.4871 rev590; local About.xml lists 1.6 support; no modVersion stated</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; local About.xml lists 1.6 support and no modVersion</x:v>
       </x:c>
       <x:c r="Q11" s="27" t="str">
         <x:v>Not runtime tested; custom storage/evidence behavior pending.</x:v>
@@ -1629,7 +1629,7 @@
         <x:v>docs/research/reviews/mods/3014915404-SmashPhil.VehicleFramework.md</x:v>
       </x:c>
       <x:c r="N12" s="27" t="str">
-        <x:v>Workshop and installed metadata reviewed; compatibility pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O12" s="27" t="str">
         <x:v>Provisional: optional vehicle interoperability only if it fits expeditions/outposts and the gravship plan.</x:v>
@@ -1682,16 +1682,16 @@
         <x:v>docs/research/reviews/mods/2574315206-imranfish.xmlextensions.md</x:v>
       </x:c>
       <x:c r="N13" s="27" t="str">
-        <x:v>Workshop and installed metadata reviewed; specific API use pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O13" s="27" t="str">
         <x:v>Provisional: optional profile tool; no Rimrooms dependency planned.</x:v>
       </x:c>
       <x:c r="P13" s="27" t="str">
-        <x:v>RimWorld 1.6.4871 rev590; local About.xml lists 1.6 support; no modVersion stated</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; local About.xml lists 1.6 support and no modVersion</x:v>
       </x:c>
       <x:c r="Q13" s="27" t="str">
-        <x:v>Not runtime tested; no custom XML Extensions use selected.</x:v>
+        <x:v>Not runtime tested; no custom XML Extension use selected.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="45" customHeight="1">
@@ -1735,10 +1735,10 @@
         <x:v>docs/research/reviews/mods/818773962-UnlimitedHugs.HugsLib.md</x:v>
       </x:c>
       <x:c r="N14" s="27" t="str">
-        <x:v>Workshop and installed metadata reviewed; compatibility pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O14" s="27" t="str">
-        <x:v>Provisional: optional profile library; no direct Rimrooms dependency planned.</x:v>
+        <x:v>Provisional: optional library for profile mods; no direct Rimrooms dependency planned.</x:v>
       </x:c>
       <x:c r="P14" s="27" t="str">
         <x:v>RimWorld 1.6.4871 rev590; local description version 12.0.0</x:v>
@@ -1788,13 +1788,13 @@
         <x:v>docs/research/reviews/mods/2023507013-OskarPotocki.VanillaFactionsExpanded.Core.md</x:v>
       </x:c>
       <x:c r="N15" s="27" t="str">
-        <x:v>Workshop and installed metadata reviewed; VGE runtime checks pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O15" s="27" t="str">
         <x:v>Provisional: required by the selected Gravship Expanded chain; optional to the Core-only Rimrooms campaign.</x:v>
       </x:c>
       <x:c r="P15" s="27" t="str">
-        <x:v>RimWorld 1.6.4871 rev590; local About.xml lists 1.6 support; no modVersion stated</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; local About.xml lists 1.6 support and no modVersion</x:v>
       </x:c>
       <x:c r="Q15" s="27" t="str">
         <x:v>Not runtime tested; clean VGE and combined-profile checks pending.</x:v>
@@ -1817,40 +1817,40 @@
         <x:v>https://steamcommunity.com/sharedfiles/filedetails/?id=3357749890</x:v>
       </x:c>
       <x:c r="F16" s="24" t="str">
-        <x:v>Materials, cargo, and recovered resources</x:v>
+        <x:v>Staff work-flow quality of life</x:v>
       </x:c>
       <x:c r="G16" s="24" t="str">
-        <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
+        <x:v>Harmony required; selected work convenience, not a Rimrooms dependency.</x:v>
       </x:c>
       <x:c r="H16" s="24" t="str">
-        <x:v>Use carrying, item handling, harvest, and salvage rules to shape expedition kit limits and recovered-cargo value. Preserve each mod's normal material and weight behavior; add only a Backrooms cargo manifest and appraisal layer.</x:v>
+        <x:v>Let players use its stump, blight, and mature-plant orders when managing facility or outpost grounds.</x:v>
       </x:c>
       <x:c r="I16" s="24" t="str">
-        <x:v>Medium: weight, stack, yield, and destruction rules affect mission capacity and valuation. Reconcile cargo accounting with item transfers and avoid duplicate salvage or recipe patches.</x:v>
+        <x:v>Keep Rimrooms roles on native work orders and avoid reassigning its designations.</x:v>
       </x:c>
       <x:c r="J16" s="24" t="str">
-        <x:v>Medium: verify stack, weight, ownership, caravan, and RWT transfer behavior for mission cargo.</x:v>
+        <x:v>Verify queued cutting/harvest jobs and overlapping plant-management mods on the selected DLC/profile.</x:v>
       </x:c>
       <x:c r="K16" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
+        <x:v>Workshop description/change notes and installed metadata reviewed; work-queue interaction pending.</x:v>
       </x:c>
       <x:c r="L16" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-FAC;RR-OUT;RR-COMPAT</x:v>
       </x:c>
       <x:c r="M16" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/3357749890-Arylice.Rimworld.AutomaticStumpChopping.md</x:v>
       </x:c>
       <x:c r="N16" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O16" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: optional job convenience; preserve existing orders and do not add a Rimrooms dependency.</x:v>
       </x:c>
       <x:c r="P16" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; Automatic Stump Chopping 1.0</x:v>
       </x:c>
       <x:c r="Q16" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; job queue and DLC plant interactions pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="45" customHeight="1">
@@ -1873,37 +1873,37 @@
         <x:v>Animals and field support</x:v>
       </x:c>
       <x:c r="G17" s="24" t="str">
-        <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
+        <x:v>Harmony required; optional animal/outpost behavior, not a Rimrooms dependency.</x:v>
       </x:c>
       <x:c r="H17" s="24" t="str">
-        <x:v>Use animals for company security, cargo, food, breeding, and field support when the installed content allows it. Keep staff hiring and mission completion viable without a particular animal species or animal mod.</x:v>
+        <x:v>Leave animal grazing and plant regrowth to the existing profile rules.</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
-        <x:v>Low to medium: respect each mod's animal, pen, medical, and apparel definitions. Check load order and travel/ownership when animals accompany expedition teams.</x:v>
+        <x:v>Do not create a second grazing system; keep outpost and facility support independent of it.</x:v>
       </x:c>
       <x:c r="J17" s="24" t="str">
-        <x:v>Low to medium: no hard dependency planned; confirm the native content works on expedition maps and stays transferable.</x:v>
+        <x:v>The page warns that other plant-ingestion changes may conflict; exact animal/plant rows still need review.</x:v>
       </x:c>
       <x:c r="K17" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
+        <x:v>Official Workshop page and installed metadata reviewed; plant/animal overlap pending.</x:v>
       </x:c>
       <x:c r="L17" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-OUT;RR-FAC;RR-COMPAT</x:v>
       </x:c>
       <x:c r="M17" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/2302739121-kittahkhan.grazeup.md</x:v>
       </x:c>
       <x:c r="N17" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O17" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: optional animal/outpost behavior; no Rimrooms dependency planned.</x:v>
       </x:c>
       <x:c r="P17" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; local About.xml lists support through 1.6; no modVersion stated</x:v>
       </x:c>
       <x:c r="Q17" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; plant-ingestion and animal-profile interactions pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="45" customHeight="1">
@@ -1926,37 +1926,37 @@
         <x:v>World operations, contracts, and commerce</x:v>
       </x:c>
       <x:c r="G18" s="24" t="str">
-        <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
+        <x:v>Harmony required; profile also has Trade Ships Drop Spot and Trade Ships No Matter What.</x:v>
       </x:c>
       <x:c r="H18" s="24" t="str">
-        <x:v>Use world events, factions, comms, traders, and saleable goods to support company contracts, procurement, outposts, and revenue. Add company jobs through a dedicated Operations interface while honoring the profile's comms and quest settings.</x:v>
+        <x:v>May help players arrange purchases; Rimrooms contracts must not assume an orbital ship can be called.</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
-        <x:v>Medium to high: world objects, quests, traders, and site creation require exact RimWorld Together synchronization review. Keep the company ledger distinct from vanilla silver and other mods' transaction state.</x:v>
+        <x:v>Leave calls and trader options on the existing Comms Console; no Rimrooms trade-ship override planned.</x:v>
       </x:c>
       <x:c r="J18" s="24" t="str">
-        <x:v>Medium to high: inspect world-object, quest, site, and RWT state ownership before adding patches.</x:v>
+        <x:v>Direct Steam page fetch was rate-limited. Combined trader type, landing spot, goods, price, cooldown, and modded-item behavior are unknown.</x:v>
       </x:c>
       <x:c r="K18" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
+        <x:v>Installed metadata and indexed official listing reviewed; full page/API/runtime evidence pending.</x:v>
       </x:c>
       <x:c r="L18" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-ECO;RR-COMPAT</x:v>
       </x:c>
       <x:c r="M18" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/3722921543-zal.calltradeships.md</x:v>
       </x:c>
       <x:c r="N18" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O18" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: optional trade convenience; no Rimrooms dependency and no contract guarantee of a called ship.</x:v>
       </x:c>
       <x:c r="P18" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; Call Trade Ships (Continued) 1.0.1</x:v>
       </x:c>
       <x:c r="Q18" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; verify with Trade Ships Drop Spot and Trade Ships No Matter What.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="45" customHeight="1">
@@ -1979,37 +1979,37 @@
         <x:v>Power and industrial infrastructure</x:v>
       </x:c>
       <x:c r="G19" s="24" t="str">
-        <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
+        <x:v>No dependency; optional map setup utility, not a Rimrooms power feature.</x:v>
       </x:c>
       <x:c r="H19" s="24" t="str">
-        <x:v>Use existing generation, switching, storage, and industrial production to build the headquarters power grid and gate reserve. Backrooms progression should add clear gate-specific operating costs and failure states without replacing the profile's power systems.</x:v>
+        <x:v>Keep generated facility/outpost maps usable without moving natural geothermal sites.</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
-        <x:v>Medium: balance and component changes can affect gate uptime. Respect profile choices that suppress vanilla events; add Backrooms-specific pressure only through its own incidents and machine state.</x:v>
+        <x:v>No Rimrooms adapter or map-generation dependency planned.</x:v>
       </x:c>
       <x:c r="J19" s="24" t="str">
-        <x:v>Medium: reconcile gate reserves and running costs with this mod's power rules; don't assume disabled vanilla events.</x:v>
+        <x:v>Publisher says it is intended for a new map; existing-map use needs God Mode.</x:v>
       </x:c>
       <x:c r="K19" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
+        <x:v>Official Workshop page and installed metadata reviewed; map behavior pending.</x:v>
       </x:c>
       <x:c r="L19" s="27" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-FAC;RR-OUT;RR-COMPAT</x:v>
       </x:c>
       <x:c r="M19" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>docs/research/reviews/mods/1547361568-LingLuo.MoveSteamGeyser.md</x:v>
       </x:c>
       <x:c r="N19" s="27" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O19" s="27" t="str">
-        <x:v>Pending review</x:v>
+        <x:v>Provisional: optional map setup utility; no Rimrooms dependency or generated-terrain reliance.</x:v>
       </x:c>
       <x:c r="P19" s="27" t="str">
-        <x:v>Not pinned</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; local metadata lists 1.0-1.6 support; no modVersion stated</x:v>
       </x:c>
       <x:c r="Q19" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Not runtime tested; new-map and existing-save behavior pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="45" customHeight="1">
@@ -16643,7 +16643,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b108bc1453f48af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab2820c6ecdd448f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: document RWT async co-op prep
</commit_message>
<xml_diff>
--- a/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
+++ b/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R33055fb13a884bd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="R15bfcc9aaae54e2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R74a09034959942c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="R11cfac814cf7453b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -82,7 +82,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -148,6 +148,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -446,7 +449,7 @@
         <x:v>Selected multiplayer model</x:v>
       </x:c>
       <x:c r="B10" s="15" t="str">
-        <x:v>Separate company branches; enable only activities verified on the pinned RWT client/server build. No live shared-map control or global company research contract.</x:v>
+        <x:v>Separate company branches; favor offline visits, supply/aid exchange, and shared investigation stories if confirmed. No shared-map control or automatic global research.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -478,7 +481,7 @@
         <x:v>Register evidence level</x:v>
       </x:c>
       <x:c r="B14" s="15" t="str">
-        <x:v>Twelve profile rows have source/metadata notes and provisional use boundaries; API/runtime checks remain open, and the other 282 entries need their first source review.</x:v>
+        <x:v>Thirteen profile rows now have source/metadata notes and provisional use boundaries; 281 remain pending. No combined-profile runtime compatibility is established.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -486,7 +489,7 @@
         <x:v>Technology exchange</x:v>
       </x:c>
       <x:c r="B15" s="15" t="str">
-        <x:v>Design a transferable Backrooms research dossier; each receiving branch studies it locally. RWT does not document built-in shared research. Confirm modded-item transfer support before enabling this feature.</x:v>
+        <x:v>Trade a Backrooms research dossier as cargo; the receiving company studies it locally. Custom-item transfer is untested; research does not unlock automatically for both branches.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -494,7 +497,7 @@
         <x:v>Facility visits</x:v>
       </x:c>
       <x:c r="B16" s="15" t="str">
-        <x:v>The Workshop description advertises visits. Exact online/offline behavior, server settings, and activity semantics are unverified; validate against the pinned release before designing features around visits.</x:v>
+        <x:v>Official RWT guidance lists offline visits and raids. Exact activity options and the visit experience remain untested on the pinned build.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -502,7 +505,7 @@
         <x:v>Current RWT boundary</x:v>
       </x:c>
       <x:c r="B17" s="15" t="str">
-        <x:v>The 294 local client/server IDs and order match, but the server does not enforce them. The Windows server archive matches the published RWT 26.8.31.1 asset; the client DLL is pinned separately. Custom transfers, visits, and scenario joining remain untested.</x:v>
+        <x:v>Local client/server IDs and order match, but the server does not enforce them. The server release and client artifact are pinned; separate starts, offline visits, supply/aid transfer, and reconnect checks remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -11393,7 +11396,7 @@
         <x:v>Not runtime tested</x:v>
       </x:c>
     </x:row>
-    <x:row r="197" ht="45" customHeight="1">
+    <x:row r="197" ht="66" hidden="0" customHeight="1">
       <x:c r="A197" s="26" t="str">
         <x:v>196</x:v>
       </x:c>
@@ -11410,40 +11413,40 @@
         <x:v>https://steamcommunity.com/sharedfiles/filedetails/?id=3005289691</x:v>
       </x:c>
       <x:c r="F197" s="24" t="str">
-        <x:v>Multiplayer: guild and world exchange</x:v>
+        <x:v>Multiplayer: separate colonies and shared-world exchange</x:v>
       </x:c>
       <x:c r="G197" s="24" t="str">
-        <x:v>Selected co-op target; optional to a solo Backrooms install. Official Workshop description advertises separate colonies and several co-op/world activities; exact runtime and transfer behavior must be verified against the pinned build.</x:v>
+        <x:v>Selected co-op target; optional to solo play. Local metadata supports RimWorld 1.5/1.6 and requires Harmony.</x:v>
       </x:c>
       <x:c r="H197" s="24" t="str">
-        <x:v>Use RWT's advertised separate-colony model for cooperative company branches. The Workshop description lists activities such as visiting, raiding, spying, trading, factions/guilds, roads, and sites. Keep company research local; enable item/pawn exchange and other actions only after testing the exact client/server build and settings.</x:v>
+        <x:v>Players run separate companies; visits, supplies, aid, and case reports can link their stories if the pinned build supports them.</x:v>
       </x:c>
       <x:c r="I197" s="24" t="str">
-        <x:v>Keep integration behind one optional adapter. Inspect the pinned release's supported APIs and settings; preserve local branch ownership, detect disabled features, and use transaction receipts only for exchanges proven to work. Do not patch server internals or assume online/offline visit behavior.</x:v>
+        <x:v>Use supported RWT activities where they fit. Keep each company's facility, gate, discoveries, research, and ledger on its own branch. Do not assume custom dossier or gear transfers.</x:v>
       </x:c>
       <x:c r="J197" s="24" t="str">
-        <x:v>High: local client/server package IDs and order match in the 2026-09-27 snapshot, but the server has AllowAllMods=true, EnforceSettings=false, ModOrder=null, and an unresolved product hash. Wiki details could not be retrieved (HTTP 403). Do not assume live control, transfer, visit, or scenario-join semantics; validate them in the pinned release.</x:v>
+        <x:v>Official docs list offline visits/raids and item/pawn exchange. The local activity settings and exact results remain untested; the server does not enforce mod order/settings.</x:v>
       </x:c>
       <x:c r="K197" s="24" t="str">
-        <x:v>Official Workshop/release pages and local profile snapshot reviewed. RWT wiki returned HTTP 403; local server release identity, exact activity semantics, runtime behavior, and Backrooms adapters remain pending.</x:v>
-      </x:c>
-      <x:c r="L197" s="27" t="str">
-        <x:v>Pending mapping</x:v>
-      </x:c>
-      <x:c r="M197" s="27" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="N197" s="27" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="O197" s="27" t="str">
-        <x:v>Pending review</x:v>
-      </x:c>
-      <x:c r="P197" s="27" t="str">
-        <x:v>Not pinned</x:v>
-      </x:c>
-      <x:c r="Q197" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Workshop/wiki/release info, local metadata, profile config, and release tree reviewed; two-player compatibility and any client extension remain unconfirmed.</x:v>
+      </x:c>
+      <x:c r="L197" s="28" t="str">
+        <x:v>RR-MP;RR-ECO;RR-COMPAT</x:v>
+      </x:c>
+      <x:c r="M197" s="28" t="str">
+        <x:v>docs/research/reviews/mods/3005289691-nova.rimworldtogether.md</x:v>
+      </x:c>
+      <x:c r="N197" s="28" t="str">
+        <x:v>Reviewed—source facts recorded</x:v>
+      </x:c>
+      <x:c r="O197" s="28" t="str">
+        <x:v>Provisional: async co-op layer for separate facilities; use offline visits/supply exchange only after pinned-build checks. No live shared-map or shared research.</x:v>
+      </x:c>
+      <x:c r="P197" s="28" t="str">
+        <x:v>RimWorld 1.6.4871 rev590; local RWT server archive matches release 26.8.31.1 asset; local client DLL hash in feasibility audit</x:v>
+      </x:c>
+      <x:c r="Q197" s="28" t="str">
+        <x:v>Not runtime tested; separate starts, offline visit, supply/aid exchange, reconnect, and custom dossier transfer pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="198" ht="45" customHeight="1">
@@ -16643,7 +16646,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab2820c6ecdd448f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bb24c9fb31d4110"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: review facility power and storage mods
</commit_message>
<xml_diff>
--- a/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
+++ b/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R74a09034959942c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="R11cfac814cf7453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rdf4c9c1e666d4718"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="R5ff16a5122bc4a69"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -476,12 +476,12 @@
         <x:v>Chapter 2 requires Odyssey, Vanilla Expanded Framework, and Chapter 1.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="24" hidden="0" customHeight="1">
       <x:c r="A14" s="14" t="str">
         <x:v>Register evidence level</x:v>
       </x:c>
       <x:c r="B14" s="15" t="str">
-        <x:v>Thirteen profile rows now have source/metadata notes and provisional use boundaries; 281 remain pending. No combined-profile runtime compatibility is established.</x:v>
+        <x:v>Seventeen profile rows have source/metadata notes; 277 remain pending. Four reviewed power/storage pages currently report Steam Community removal; no combined-profile runtime compatibility is established.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2015,7 +2015,7 @@
         <x:v>Not runtime tested; new-map and existing-save behavior pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="45" customHeight="1">
+    <x:row r="20" ht="66" hidden="0" customHeight="1">
       <x:c r="A20" s="26" t="str">
         <x:v>19</x:v>
       </x:c>
@@ -2035,37 +2035,37 @@
         <x:v>Power and industrial infrastructure</x:v>
       </x:c>
       <x:c r="G20" s="24" t="str">
-        <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
+        <x:v>Selected profile utility; optional to Rimrooms Core. Local metadata lists RimWorld 1.6 support.</x:v>
       </x:c>
       <x:c r="H20" s="24" t="str">
-        <x:v>Use existing generation, switching, storage, and industrial production to build the headquarters power grid and gate reserve. Backrooms progression should add clear gate-specific operating costs and failure states without replacing the profile's power systems.</x:v>
+        <x:v>Potential control-room model for switching facility power zones; keep the gate usable without it.</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
-        <x:v>Medium: balance and component changes can affect gate uptime. Respect profile choices that suppress vanilla events; add Backrooms-specific pressure only through its own incidents and machine state.</x:v>
+        <x:v>Preserve the mod's own remote toggle, if verified. Do not replace vanilla switches or assume automatic control.</x:v>
       </x:c>
       <x:c r="J20" s="24" t="str">
-        <x:v>Medium: reconcile gate reserves and running costs with this mod's power rules; don't assume disabled vanilla events.</x:v>
+        <x:v>Workshop page currently reports removal; local copy is installed. Publisher notes a soft conflict with Auto Flicker, absent from this profile.</x:v>
       </x:c>
       <x:c r="K20" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
-      </x:c>
-      <x:c r="L20" s="27" t="str">
-        <x:v>Pending mapping</x:v>
-      </x:c>
-      <x:c r="M20" s="27" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="N20" s="27" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="O20" s="27" t="str">
-        <x:v>Pending review</x:v>
-      </x:c>
-      <x:c r="P20" s="27" t="str">
-        <x:v>Not pinned</x:v>
-      </x:c>
-      <x:c r="Q20" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Workshop page and local About.xml reviewed; both list RimWorld 1.4–1.6 support; no runtime test.</x:v>
+      </x:c>
+      <x:c r="L20" s="28" t="str">
+        <x:v>RR-FAC;RR-GATE;RR-COMPAT</x:v>
+      </x:c>
+      <x:c r="M20" s="28" t="str">
+        <x:v>docs/research/reviews/mods/3031634496-Og.AutomaticPowerSwitch.md</x:v>
+      </x:c>
+      <x:c r="N20" s="28" t="str">
+        <x:v>Reviewed—source facts recorded</x:v>
+      </x:c>
+      <x:c r="O20" s="28" t="str">
+        <x:v>Provisional: optional facility power-control convenience; do not require or repackage it. Steam page currently reports removal; local profile copy is installed.</x:v>
+      </x:c>
+      <x:c r="P20" s="28" t="str">
+        <x:v>RimWorld 1.6.4871 rev590; local About.xml supports 1.4, 1.5, and 1.6; Workshop page advertises same</x:v>
+      </x:c>
+      <x:c r="Q20" s="28" t="str">
+        <x:v>Not runtime tested; remote switch, Microelectronics unlock, save/reload, and named Auto Flicker conflict checks pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="45" customHeight="1">
@@ -2280,7 +2280,7 @@
         <x:v>Not runtime tested</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="45" customHeight="1">
+    <x:row r="25" ht="66" hidden="0" customHeight="1">
       <x:c r="A25" s="26" t="str">
         <x:v>24</x:v>
       </x:c>
@@ -2300,40 +2300,40 @@
         <x:v>Storage and recovered-material logistics</x:v>
       </x:c>
       <x:c r="G25" s="24" t="str">
-        <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
+        <x:v>Selected profile entry; optional to Core. Requires Ideology DLC and Adaptive Storage Framework.</x:v>
       </x:c>
       <x:c r="H25" s="24" t="str">
-        <x:v>Use existing storage, hauling, and refrigeration for expedition kits, sample quarantine, evidence archives, food, and sale stock. Add Backrooms labels and custody rules through separate definitions rather than global storage rewrites.</x:v>
+        <x:v>Optional ideology-themed storage furniture for archive, relic, or ceremonial rooms.</x:v>
       </x:c>
       <x:c r="I25" s="24" t="str">
-        <x:v>Medium: confirm filters and stack rules can distinguish quarantined samples, ordinary stock, and mission cargo. Avoid patches that overwrite other storage mods' categories.</x:v>
+        <x:v>Use only when both Ideology and Adaptive Storage Framework are present; keep ordinary Core storage available.</x:v>
       </x:c>
       <x:c r="J25" s="24" t="str">
-        <x:v>Medium: verify stack, weight, ownership, caravan, and RWT transfer behavior for mission cargo.</x:v>
+        <x:v>Workshop page currently reports removal. Publisher names third-party art/content; do not copy the module's files.</x:v>
       </x:c>
       <x:c r="K25" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
-      </x:c>
-      <x:c r="L25" s="27" t="str">
-        <x:v>Pending mapping</x:v>
-      </x:c>
-      <x:c r="M25" s="27" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="N25" s="27" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="O25" s="27" t="str">
-        <x:v>Pending review</x:v>
-      </x:c>
-      <x:c r="P25" s="27" t="str">
-        <x:v>Not pinned</x:v>
-      </x:c>
-      <x:c r="Q25" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="45" customHeight="1">
+        <x:v>Workshop page and local About.xml reviewed; supports RimWorld 1.4–1.6; requires Ideology and Adaptive Storage Framework.</x:v>
+      </x:c>
+      <x:c r="L25" s="28" t="str">
+        <x:v>RR-FAC;RR-EVD;RR-DLC;RR-COMPAT</x:v>
+      </x:c>
+      <x:c r="M25" s="28" t="str">
+        <x:v>docs/research/reviews/mods/3301337278-Adaptive.Ideology.Storage.md</x:v>
+      </x:c>
+      <x:c r="N25" s="28" t="str">
+        <x:v>Reviewed—source facts recorded</x:v>
+      </x:c>
+      <x:c r="O25" s="28" t="str">
+        <x:v>Provisional: optional Ideology and Adaptive Storage Framework furniture storage; keep archive/evidence storage available on Core. Steam page currently reports removal.</x:v>
+      </x:c>
+      <x:c r="P25" s="28" t="str">
+        <x:v>RimWorld 1.6.4871 rev590; local About.xml supports 1.4, 1.5, and 1.6; requires Ideology and Adaptive Storage Framework</x:v>
+      </x:c>
+      <x:c r="Q25" s="28" t="str">
+        <x:v>Not runtime tested; DLC-absent safety, storage filters, trade visibility, and selected-profile behavior pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A26" s="26" t="str">
         <x:v>25</x:v>
       </x:c>
@@ -2353,40 +2353,40 @@
         <x:v>Storage and recovered-material logistics</x:v>
       </x:c>
       <x:c r="G26" s="24" t="str">
-        <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
+        <x:v>Selected profile entry; optional to Core. Requires Adaptive Storage Framework; local metadata also lists Harmony.</x:v>
       </x:c>
       <x:c r="H26" s="24" t="str">
-        <x:v>Use existing storage, hauling, and refrigeration for expedition kits, sample quarantine, evidence archives, food, and sale stock. Add Backrooms labels and custody rules through separate definitions rather than global storage rewrites.</x:v>
+        <x:v>Optional rough racks, piles, and cellars for stores, kitchens, field kits, and outposts.</x:v>
       </x:c>
       <x:c r="I26" s="24" t="str">
-        <x:v>Medium: confirm filters and stack rules can distinguish quarantined samples, ordinary stock, and mission cargo. Avoid patches that overwrite other storage mods' categories.</x:v>
+        <x:v>Keep sample and food records separate from furniture. Test cellar food-preservation claims before relying on them.</x:v>
       </x:c>
       <x:c r="J26" s="24" t="str">
-        <x:v>Medium: verify stack, weight, ownership, caravan, and RWT transfer behavior for mission cargo.</x:v>
+        <x:v>Workshop page currently reports removal. Publisher notes cellar temperature limits; do not copy the module's art or code.</x:v>
       </x:c>
       <x:c r="K26" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
-      </x:c>
-      <x:c r="L26" s="27" t="str">
-        <x:v>Pending mapping</x:v>
-      </x:c>
-      <x:c r="M26" s="27" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="N26" s="27" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="O26" s="27" t="str">
-        <x:v>Pending review</x:v>
-      </x:c>
-      <x:c r="P26" s="27" t="str">
-        <x:v>Not pinned</x:v>
-      </x:c>
-      <x:c r="Q26" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="45" customHeight="1">
+        <x:v>Workshop page and local About.xml reviewed; page supports RimWorld 1.5/1.6; local metadata lists Harmony and Adaptive Storage Framework.</x:v>
+      </x:c>
+      <x:c r="L26" s="28" t="str">
+        <x:v>RR-FAC;RR-EVD;RR-OUT;RR-COMPAT</x:v>
+      </x:c>
+      <x:c r="M26" s="28" t="str">
+        <x:v>docs/research/reviews/mods/3400037215-Adaptive.PrimitiveStorage.md</x:v>
+      </x:c>
+      <x:c r="N26" s="28" t="str">
+        <x:v>Reviewed—source facts recorded</x:v>
+      </x:c>
+      <x:c r="O26" s="28" t="str">
+        <x:v>Provisional: optional field, food, and rough-outpost storage; treat cellar preservation as unverified. Steam page currently reports removal.</x:v>
+      </x:c>
+      <x:c r="P26" s="28" t="str">
+        <x:v>RimWorld 1.6.4871 rev590; local About.xml supports 1.5/1.6 and lists Harmony plus Adaptive Storage Framework</x:v>
+      </x:c>
+      <x:c r="Q26" s="28" t="str">
+        <x:v>Not runtime tested; cellar temperatures/food decay, storage filters, trade visibility, and save/reload pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A27" s="26" t="str">
         <x:v>26</x:v>
       </x:c>
@@ -2406,37 +2406,37 @@
         <x:v>Storage and recovered-material logistics</x:v>
       </x:c>
       <x:c r="G27" s="24" t="str">
-        <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
+        <x:v>Selected profile entry; optional to Core. Requires Adaptive Storage Framework.</x:v>
       </x:c>
       <x:c r="H27" s="24" t="str">
-        <x:v>Use existing storage, hauling, and refrigeration for expedition kits, sample quarantine, evidence archives, food, and sale stock. Add Backrooms labels and custody rules through separate definitions rather than global storage rewrites.</x:v>
+        <x:v>Optional crates, racks, and cabinets for equipment stores, evidence archives, and shipping rooms.</x:v>
       </x:c>
       <x:c r="I27" s="24" t="str">
-        <x:v>Medium: confirm filters and stack rules can distinguish quarantined samples, ordinary stock, and mission cargo. Avoid patches that overwrite other storage mods' categories.</x:v>
+        <x:v>Keep custody and evidence records separate from the containers; preserve ordinary storage if the module is absent.</x:v>
       </x:c>
       <x:c r="J27" s="24" t="str">
-        <x:v>Medium: verify stack, weight, ownership, caravan, and RWT transfer behavior for mission cargo.</x:v>
+        <x:v>Workshop page currently reports removal. Publisher documents an older update that could hide containers; stored items were reported safe.</x:v>
       </x:c>
       <x:c r="K27" s="24" t="str">
-        <x:v>Local name/ID record reviewed and mapped to a design family; exact Workshop page, dependency, source behavior, and compatibility remain pending unless separately cited.</x:v>
-      </x:c>
-      <x:c r="L27" s="27" t="str">
-        <x:v>Pending mapping</x:v>
-      </x:c>
-      <x:c r="M27" s="27" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="N27" s="27" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="O27" s="27" t="str">
-        <x:v>Pending review</x:v>
-      </x:c>
-      <x:c r="P27" s="27" t="str">
-        <x:v>Not pinned</x:v>
-      </x:c>
-      <x:c r="Q27" s="27" t="str">
-        <x:v>Not runtime tested</x:v>
+        <x:v>Workshop page and local About.xml reviewed; supports RimWorld 1.4–1.6; requires Adaptive Storage Framework.</x:v>
+      </x:c>
+      <x:c r="L27" s="28" t="str">
+        <x:v>RR-FAC;RR-EVD;RR-COMPAT</x:v>
+      </x:c>
+      <x:c r="M27" s="28" t="str">
+        <x:v>docs/research/reviews/mods/3297307747-Adaptive.SimpleStorage.md</x:v>
+      </x:c>
+      <x:c r="N27" s="28" t="str">
+        <x:v>Reviewed—source facts recorded</x:v>
+      </x:c>
+      <x:c r="O27" s="28" t="str">
+        <x:v>Provisional: optional crate, rack, and cabinet storage for facility rooms; preserve ordinary storage if absent. Steam page currently reports removal.</x:v>
+      </x:c>
+      <x:c r="P27" s="28" t="str">
+        <x:v>RimWorld 1.6.4871 rev590; local About.xml supports 1.4, 1.5, and 1.6; requires Adaptive Storage Framework</x:v>
+      </x:c>
+      <x:c r="Q27" s="28" t="str">
+        <x:v>Not runtime tested; construction, hauling/bills, trade visibility, and save/reload with the installed module remain pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="45" customHeight="1">
@@ -16646,7 +16646,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bb24c9fb31d4110"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R010e5cc9450e4595"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: finish 294 source review intake
</commit_message>
<xml_diff>
--- a/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
+++ b/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4d15b45f42b84f25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="Rc4587ff3a2054ef9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R92966c98affc4df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="R0908af074b97493a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -481,7 +481,7 @@
         <x:v>Register evidence level</x:v>
       </x:c>
       <x:c r="B14" s="15" t="str">
-        <x:v>291 of 294 rows have accepted source-fact records; 3 remain pending. Partial source notes: rows 96, 237, and 278. No combined-profile compatibility is established by source review.</x:v>
+        <x:v>All 294 of 294 rows have accepted source-fact records with known limits recorded; no combined-profile runtime clearance has been established.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -505,7 +505,7 @@
         <x:v>Current RWT boundary</x:v>
       </x:c>
       <x:c r="B17" s="15" t="str">
-        <x:v>Local client/server IDs and order match, but the server does not enforce them. The server release and client artifact are pinned; separate starts, offline visits, supply/aid transfer, and reconnect checks remain pending.</x:v>
+        <x:v>Local client/server IDs and order match. The RWT 26.8.31.1 server archive matches the official release digest; the client artifact is pinned separately by hash. Server settings do not enforce the profile. Visits, custom cargo, differing scenarios, and reconnect behavior remain untested.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -4020,7 +4020,7 @@
         <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O57" s="28" t="str">
-        <x:v>Provisional: optional profile QoL; no Rimrooms feature requires this mod. Keep native behavior untouched; 1.6 full-profile check pending.</x:v>
+        <x:v>Optional profile entry; preserve native milkable-animal behavior; no Rimrooms feature depends on it. Do not claim 1.6 compatibility from the local About.xml, which omits 1.6.</x:v>
       </x:c>
       <x:c r="P57" s="28" t="str">
         <x:v>RimWorld 1.6.4871 rev590; local About.xml omits 1.6; no modVersion; About.xml SHA256 2979A22559220FACF843F4E0600488958D1DC94CC8F6CE7B0329985E9E3B865E</x:v>
@@ -6119,16 +6119,16 @@
         <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
       </x:c>
       <x:c r="H97" s="24" t="str">
-        <x:v>Use fueled cremation as an optional company procedure for dangerous remains, contaminated waste, and post-incident cleanup; leave disposition to player policy.</x:v>
+        <x:v>Optional company procedure for ordinary remains and facility waste. Preserve Rimrooms evidence custody, sample analysis, and case disposition before any destruction.</x:v>
       </x:c>
       <x:c r="I97" s="24" t="str">
-        <x:v>Low to medium: verify corpse, prisoner, and evidence custody rules before offering a custom cleanup job.</x:v>
+        <x:v>No direct Rimrooms adapter or patch. Retain native cremation bills and recipes where present; use this as an optional facility example only.</x:v>
       </x:c>
       <x:c r="J97" s="24" t="str">
-        <x:v>Medium: check pawn health/custody state, treatment choice, and transfer; preserve a vanilla fallback.</x:v>
+        <x:v>Publisher lists RimWorld 1.5/1.6 and optional patches for Rim of Madness – Bones and Ashes. These are patch targets, not required dependencies. Check fuel, bills, corpse contents, destruction, and row 152 interactions before runtime claims.</x:v>
       </x:c>
       <x:c r="K97" s="24" t="str">
-        <x:v>Source review incomplete; direct publisher-source check pending.</x:v>
+        <x:v>Publisher and local source facts recorded; Rimrooms runtime compatibility pending.</x:v>
       </x:c>
       <x:c r="L97" s="28" t="str">
         <x:v>RR-FAC;RR-EVD;RR-THREAT;RR-COMPAT</x:v>
@@ -6137,16 +6137,16 @@
         <x:v>docs/research/reviews/mods/3286907608-Xercaine.FueledCrematorium.md</x:v>
       </x:c>
       <x:c r="N97" s="28" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O97" s="28" t="str">
-        <x:v>Pending primary-source review; provisional optional disposal furniture, never an evidence workflow.</x:v>
+        <x:v>Optional; no direct integration. Preserve evidence custody before destruction; profile and RWT coexistence are not runtime-verified.</x:v>
       </x:c>
       <x:c r="P97" s="28" t="str">
-        <x:v>RimWorld 1.6.4871 rev590; local version ''; local support 1.5, 1.6; About.xml SHA-256 3E2AF3B20B59F94757902F691179A88D94B23CC7961CA4EC62549D2CA010E87E</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; local package Xercaine.FueledCrematorium; supports 1.5/1.6; no local modVersion; About.xml SHA-256 3E2AF3B20B59F94757902F691179A88D94B23CC7961CA4EC62549D2CA010E87E</x:v>
       </x:c>
       <x:c r="Q97" s="28" t="str">
-        <x:v>Wave 11 exact and English-page retries still rate-limited; no publisher-linked source/license verified. Existing indexed description remains unconfirmed; no runtime test.</x:v>
+        <x:v>Publisher page via alternate exact-ID route and author comments checked 2026-09-27; local 1.6 XML checked. No source repository/license found. Steam removal/generic incompatibility banners are page state, not runtime findings. No runtime test.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="45" customHeight="1">
@@ -10698,13 +10698,13 @@
         <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O183" s="28" t="str">
-        <x:v>Provisional: solo-only optional pending Gate 0 choice; publisher says multiplayer will not work properly.</x:v>
+        <x:v>Optional; include in the owner-selected RWT candidate test profile despite the publisher multiplayer warning; do not advertise co-op support before exact-profile results.</x:v>
       </x:c>
       <x:c r="P183" s="28" t="str">
         <x:v>RimWorld 1.6.4871 rev590; local version 1.6.5; supports 1.0-1.6; Harmony required; upstream repository lists MIT; About SHA-256 07A3C667B6B6729378D4EEDD5CACDBCC5F87A74B72546875D8ACD112CF982033</x:v>
       </x:c>
       <x:c r="Q183" s="28" t="str">
-        <x:v>Not runtime tested; verify Hospitality vat performance, medical/prisoner overlap, and exact RWT profile before support.</x:v>
+        <x:v>Publisher warns multiplayer may not work properly. Owner selected this row for RWT candidate testing on 2026-09-27; no runtime test or RWT support clearance yet. Verify Hospitality, medical/prisoner overlap, and desync behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="184" ht="45" customHeight="1">
@@ -13592,34 +13592,34 @@
         <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
       </x:c>
       <x:c r="H238" s="24" t="str">
-        <x:v>Use the active trait, memory, social-fight, relationship, conversion, and faction-reaction rules when generating applicants, workplace incidents, and crew histories. Keep the company's evaluation based on actual pawn traits, skills, and relationships.</x:v>
+        <x:v>Account for this optional change to vanilla social-fight stopping conditions when resolving staff injuries, relationship conflicts, and casualties. No Rimrooms-specific behavior is demonstrated.</x:v>
       </x:c>
       <x:c r="I238" s="24" t="str">
-        <x:v>Medium: these mods change the staff and visitor experience. Avoid replacing their thought, relation, or faction logic; check how hostility and guest incidents affect company reputation.</x:v>
+        <x:v>No direct integration; leave native social-fight logic intact and keep Rimrooms staff/case records separate.</x:v>
       </x:c>
       <x:c r="J238" s="24" t="str">
-        <x:v>Low to medium: preserve native jobs, needs, guest/faction ownership, and social behavior; test custom role suggestions around them.</x:v>
+        <x:v>Publisher describes pain/injury and relationship stop checks; Masochists ignore the pain check and Bloodlust pawns can continue until surrender, death, or downing. Steam also shows generic removal and incompatibility banners without a stated reason; do not treat those as a reproduced co-op conflict.</x:v>
       </x:c>
       <x:c r="K238" s="24" t="str">
-        <x:v>Source review incomplete; direct publisher-source check pending.</x:v>
+        <x:v>Publisher and local source facts recorded; social-fight, full-profile, and RWT behavior remain runtime-pending.</x:v>
       </x:c>
       <x:c r="L238" s="28" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-STA;RR-COMPAT</x:v>
       </x:c>
       <x:c r="M238" s="28" t="str">
         <x:v>docs/research/reviews/mods/1542424705-marvinkosh.ughyougotme.md</x:v>
       </x:c>
       <x:c r="N238" s="28" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O238" s="28" t="str">
-        <x:v>Pending: direct publisher behavior and license not verified; no integration.</x:v>
+        <x:v>Optional; no direct integration. Social-fight and RWT coexistence are unverified; do not claim profile compatibility without testing.</x:v>
       </x:c>
       <x:c r="P238" s="28" t="str">
-        <x:v>Local metadata snapshot dated 2026-09-27; Version blank; local support 1.0–1.6; Harmony required and ordered after Harmony; no runtime check.</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; package marvinkosh.ughyougotme; local version blank; publisher lists 1.0.7 updated 2025-06-21 and support 1.0–1.6; Harmony required and loaded before mod.</x:v>
       </x:c>
       <x:c r="Q238" s="28" t="str">
-        <x:v>Wave 11 exact and English-page retries returned HTTP 429; old publisher site inaccessible and no linked source/license verified. Secondary references insufficient; no runtime test.</x:v>
+        <x:v>Exact publisher page, change notes, comments, and local metadata checked 2026-09-27. No source repository/license identified. Steam removal/incompatibility banners do not establish technical incompatibility. No runtime test.</x:v>
       </x:c>
     </x:row>
     <x:row r="239" ht="45" customHeight="1">
@@ -15574,13 +15574,13 @@
         <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O275" s="28" t="str">
-        <x:v>Provisional: solo-only optional recommended; RWT co-op scope awaits owner input.</x:v>
+        <x:v>Optional; include in the owner-selected RWT candidate test profile despite the publisher multiplayer/desync warning; do not advertise co-op support before exact-profile results.</x:v>
       </x:c>
       <x:c r="P275" s="28" t="str">
         <x:v>RimWorld 1.6.4871 rev590; local version ''; local support 1.0, 1.1, 1.2, 1.3, 1.4, 1.5, 1.6; About.xml SHA-256 2462E577F12FC4ED84B1CEC0118A258883194A5468C74143302B571F5A4F427E</x:v>
       </x:c>
       <x:c r="Q275" s="28" t="str">
-        <x:v>Publisher multiplayer/desync warning; no RWT test run. Owner scope requested 2026-09-27; keep outside RWT support claim pending answer and evidence.</x:v>
+        <x:v>Publisher warns multiplayer is unsupported and may desynchronize. Owner selected this row for RWT candidate testing on 2026-09-27; no runtime test or RWT support clearance yet. Test medical, custody, corpse and Harvest Organs interactions.</x:v>
       </x:c>
     </x:row>
     <x:row r="276" ht="45" customHeight="1">
@@ -15759,40 +15759,40 @@
         <x:v>https://steamcommunity.com/sharedfiles/filedetails/?id=3093303048</x:v>
       </x:c>
       <x:c r="F279" s="24" t="str">
-        <x:v>Unverified package scope — title only</x:v>
+        <x:v>Facility construction and material access</x:v>
       </x:c>
       <x:c r="G279" s="24" t="str">
         <x:v>Included in the user-selected 294-entry profile; not a Backrooms core dependency.</x:v>
       </x:c>
       <x:c r="H279" s="24" t="str">
-        <x:v>Do not plan a feature integration from the title or local load-order metadata alone.</x:v>
+        <x:v>Optional placement fix for cooler and vent construction with Replace Stuff; it restores checks against blocked intakes/exhausts and over-wall placement.</x:v>
       </x:c>
       <x:c r="I279" s="24" t="str">
-        <x:v>No integration decision until publisher feature scope and license are accessible.</x:v>
+        <x:v>No direct Rimrooms integration. Let the optional patch preserve its native placement rules; do not replace cooler/vent geometry in Rimrooms.</x:v>
       </x:c>
       <x:c r="J279" s="24" t="str">
-        <x:v>Publisher page retries were rate-limited. Local metadata declares hard dependencies on Harmony and Replace Stuff Continued, and a LoadAfter target for Replace Stuff Compatibility; that target is not declared as a hard dependency.</x:v>
+        <x:v>Hard dependencies are Harmony and Replace Stuff Continued. Local metadata orders after Garethp.ReplaceStuffCompatibility, which is absent from the profile. Publisher comments contain an unresolved pawns-fire-through-coolers report; it was not reproduced.</x:v>
       </x:c>
       <x:c r="K279" s="24" t="str">
-        <x:v>Source review incomplete; direct publisher-source check pending.</x:v>
+        <x:v>Publisher and local source facts recorded; placement and line-of-fire behavior remain runtime-pending.</x:v>
       </x:c>
       <x:c r="L279" s="28" t="str">
-        <x:v>Pending mapping</x:v>
+        <x:v>RR-FAC;RR-COMPAT</x:v>
       </x:c>
       <x:c r="M279" s="28" t="str">
         <x:v>docs/research/reviews/mods/3093303048-Deadmano.ReplaceStuffCoolerVentPlacementFix.md</x:v>
       </x:c>
       <x:c r="N279" s="28" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Reviewed—source facts recorded</x:v>
       </x:c>
       <x:c r="O279" s="28" t="str">
-        <x:v>Pending: no verified feature description or license; no integration.</x:v>
+        <x:v>Optional; no direct integration. Do not claim profile/RWT coexistence until placement and the reported line-of-fire issue are checked.</x:v>
       </x:c>
       <x:c r="P279" s="28" t="str">
-        <x:v>Local metadata snapshot dated 2026-09-27; v1.6.0; support 1.4–1.6; hard deps Harmony and Replace Stuff Continued (Memegoddess.ReplaceStuff); after Garethp.ReplaceStuffCompatibility, absent.</x:v>
+        <x:v>RimWorld 1.6.4871 rev590; package Deadmano.ReplaceStuffCoolerVentPlacementFix v1.6.0; supports 1.4–1.6; requires Harmony and Memegoddess.ReplaceStuff; loads after Garethp.ReplaceStuffCompatibility per local metadata.</x:v>
       </x:c>
       <x:c r="Q279" s="28" t="str">
-        <x:v>Exact page and alternate URL returned HTTP 429; no publisher text, linked repository, or license verified. Local metadata only; no runtime test.</x:v>
+        <x:v>Exact publisher page, change notes, comments and local metadata checked 2026-09-27. No source repository/license found. Author's continuation preference is not a general license. Pawn-fire-through-coolers report is unverified. No runtime test.</x:v>
       </x:c>
     </x:row>
     <x:row r="280" ht="45" customHeight="1">
@@ -16646,7 +16646,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra25c823537174157"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8a5db6044d34198"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: complete feature traceability and style brief
</commit_message>
<xml_diff>
--- a/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
+++ b/outputs/rimrooms-async-industries-register-2026-09-27/Rimrooms_Async_Industries_294_Mod_Integration_Register.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R92966c98affc4df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="R0908af074b97493a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rad5cc2ad2cae4118"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mod Register" sheetId="2" r:id="R607367d691144eea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4980,7 +4980,7 @@
         <x:v>RimWorld 1.6.4871 rev590; local Mlie.DingOnGameLoaded 1.6.1 / support 1.1–1.6; exact-ID indexed Workshop text checked 2026-09-27; direct Steam fetch rate-limited; no runtime test.</x:v>
       </x:c>
       <x:c r="Q75" s="28" t="str">
-        <x:v>Linked note records the indexed publisher claims and local metadata. Direct page, client audio timing, and compatibility were not tested.</x:v>
+        <x:v>Not runtime tested. Linked note records the indexed publisher claims and local metadata. Direct page, client audio timing, and compatibility were not tested.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="45" customHeight="1">
@@ -5192,7 +5192,7 @@
         <x:v>RimWorld 1.6.4871 rev590; local package metadata and indexed exact-ID publisher text checked 2026-09-27; direct page errored; not runtime tested.</x:v>
       </x:c>
       <x:c r="Q79" s="28" t="str">
-        <x:v>Permission to update is not a license grant. Animal Weapon wording and full-profile command behavior remain uncertain.</x:v>
+        <x:v>Not runtime tested. Permission to update is not a license grant. Animal Weapon wording and full-profile command behavior remain uncertain.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="45" customHeight="1">
@@ -6040,7 +6040,7 @@
         <x:v>RimWorld 1.6.4871 rev590; local selected package metadata and exact Workshop/source checked 2026-09-27; not runtime tested.</x:v>
       </x:c>
       <x:c r="Q95" s="28" t="str">
-        <x:v>Selected package is Zed item 2958300354; separate continuation 3261498531 excluded from claims. Source license and surgery behavior remain unresolved.</x:v>
+        <x:v>Not runtime tested. Selected package is Zed item 2958300354; separate continuation 3261498531 excluded from claims. Source license and surgery behavior remain unresolved.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="45" customHeight="1">
@@ -13036,7 +13036,7 @@
         <x:v>RimWorld 1.6.4871 rev590; selected local package metadata and selected/original Workshop pages checked 2026-09-27; not runtime tested.</x:v>
       </x:c>
       <x:c r="Q227" s="28" t="str">
-        <x:v>Selected-versus-original boundary and rights uncertainty recorded. Exact selected payload and cooling behavior must be verified before reliance.</x:v>
+        <x:v>Not runtime tested. Selected-versus-original boundary and rights uncertainty recorded. Exact selected payload and cooling behavior must be verified before reliance.</x:v>
       </x:c>
     </x:row>
     <x:row r="228" ht="45" customHeight="1">
@@ -16646,7 +16646,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8a5db6044d34198"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2579a00438a471e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>